<commit_message>
feat: complete 26 leather jackets with OpenCode Go DeepSeek 4.1 Flash brand & sizing extraction
</commit_message>
<xml_diff>
--- a/taobao_leather_jackets_summary.xlsx
+++ b/taobao_leather_jackets_summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="137">
   <si>
     <t>순번</t>
   </si>
@@ -37,55 +37,61 @@
     <t>저장폴더</t>
   </si>
   <si>
-    <t>811036195091</t>
-  </si>
-  <si>
-    <t>1080043211319</t>
-  </si>
-  <si>
-    <t>1083932831050</t>
-  </si>
-  <si>
-    <t>1071816497728</t>
-  </si>
-  <si>
-    <t>1075139885104</t>
-  </si>
-  <si>
-    <t>1078567805117</t>
-  </si>
-  <si>
-    <t>1061875162656</t>
-  </si>
-  <si>
-    <t>1069955447343</t>
-  </si>
-  <si>
-    <t>1075374113206</t>
-  </si>
-  <si>
-    <t>1081695145771</t>
-  </si>
-  <si>
-    <t>1054456462690</t>
-  </si>
-  <si>
-    <t>1055642429134</t>
-  </si>
-  <si>
-    <t>1062441766322</t>
-  </si>
-  <si>
-    <t>1071811849639</t>
-  </si>
-  <si>
-    <t>1073332440807</t>
-  </si>
-  <si>
-    <t>1074826657600</t>
-  </si>
-  <si>
-    <t>1075294704720</t>
+    <t>1082717808296</t>
+  </si>
+  <si>
+    <t>963160907330</t>
+  </si>
+  <si>
+    <t>1080314843824</t>
+  </si>
+  <si>
+    <t>982964565711</t>
+  </si>
+  <si>
+    <t>970351720471</t>
+  </si>
+  <si>
+    <t>1078044637886</t>
+  </si>
+  <si>
+    <t>1079411133222</t>
+  </si>
+  <si>
+    <t>1080314063229</t>
+  </si>
+  <si>
+    <t>967752064868</t>
+  </si>
+  <si>
+    <t>738083059484</t>
+  </si>
+  <si>
+    <t>1077843058059</t>
+  </si>
+  <si>
+    <t>1081834756981</t>
+  </si>
+  <si>
+    <t>1076140587381</t>
+  </si>
+  <si>
+    <t>1076689119808</t>
+  </si>
+  <si>
+    <t>1081837888025</t>
+  </si>
+  <si>
+    <t>1082130592462</t>
+  </si>
+  <si>
+    <t>680877999136</t>
+  </si>
+  <si>
+    <t>742216959144</t>
+  </si>
+  <si>
+    <t>758951256874</t>
   </si>
   <si>
     <t>vintage古着皮衣 男士修身机车款头层绵羊皮真皮外套时尚夹克 E1</t>
@@ -142,6 +148,63 @@
     <t>vintage古着皮衣 男士修身机车款头层绵羊皮真皮外套时尚夹克 X91</t>
   </si>
   <si>
+    <t>vintage古着皮衣 复古机车风美式经典皮夹克头层牛皮外套男士V154</t>
+  </si>
+  <si>
+    <t>vintage古着皮衣 复古重工头层牛皮西部印第安流苏夹克外套 V2</t>
+  </si>
+  <si>
+    <t>vintage古着皮衣 水貂毛皮草冬季外套整貂大翻领夹克双面可穿V161</t>
+  </si>
+  <si>
+    <t>vintage古着皮衣 复古吉普赛长袖流苏摩托车男士皮夹克外套 V64</t>
+  </si>
+  <si>
+    <t>vintage古着皮衣 复古吉普赛长袖流苏摩托车男士皮夹克外套W28</t>
+  </si>
+  <si>
+    <t>vintage古着皮衣 美式A2复古短款宽松飞行员皮夹克外套男女 V82</t>
+  </si>
+  <si>
+    <t>vintage古着皮衣 美式复古短款斜拉链机车服皮夹克摩托车外套V99</t>
+  </si>
+  <si>
+    <t>vintage古着皮衣 水貂毛皮草冬季外套整貂大翻领夹克双面可穿V160</t>
+  </si>
+  <si>
+    <t>vintage古着皮衣 复古磨砂牛皮西部印第安流苏摩托车夹克外套W25</t>
+  </si>
+  <si>
+    <t>vintage古着皮衣 美式复古休闲款夹克外套阿美咔叽男款 鹿皮U22</t>
+  </si>
+  <si>
+    <t>vintage古着皮衣 美式复古短款斜拉链机车服皮夹克摩托车外套V93</t>
+  </si>
+  <si>
+    <t>vintage古着皮衣 复古美式短款拉链款机车服皮夹克摩托车外套V100</t>
+  </si>
+  <si>
+    <t>vintage古着皮衣 美式A2复古短款宽松飞行员皮夹克外套男女 V80</t>
+  </si>
+  <si>
+    <t>vintage古着皮衣 美式A2复古短款宽松飞行员皮夹克外套男女 V87</t>
+  </si>
+  <si>
+    <t>vintage古着皮衣 美式休闲拉链款机车服皮夹克摩托车真皮外套V102</t>
+  </si>
+  <si>
+    <t>vintage古着皮衣 美式休闲拉链款机车服皮夹克摩托车真皮外套V103</t>
+  </si>
+  <si>
+    <t>vintage古着皮衣 复古美式休闲刺绣贴布棒球服宽松空军夹克外套14</t>
+  </si>
+  <si>
+    <t>vintage古着皮衣 美式休闲刺绣贴布棒球服宽松夹克真皮外套V246</t>
+  </si>
+  <si>
+    <t>vintage古着皮衣 美式休闲拉链款机车服皮夹克摩托车真皮外套W425</t>
+  </si>
+  <si>
     <t>https://item.taobao.com/item.htm?id=1077196468019&amp;mi_id=0000ny7GAY_eEA-5pJCJ2HRuEtR2_54HNgGqTP-gorvJQgw&amp;spm=a21xtw.29978518.0.0&amp;xxc=shop&amp;sku_properties=20509%3A838956228</t>
   </si>
   <si>
@@ -196,6 +259,63 @@
     <t>https://item.taobao.com/item.htm?id=1075294704720&amp;mi_id=0000kNLzud7RxYJJ74YArP6fzyMFnUY5AxxpuNq4NHnVTTM&amp;spm=a21xtw.29178619.0.0&amp;xxc=shop</t>
   </si>
   <si>
+    <t>https://item.taobao.com/item.htm?id=1082717808296&amp;mi_id=0000sQhOtNhpDhJ1tGlaJEqrmXoSO6ADaZmth7MWl4S1wP4&amp;spm=a21xtw.29978516.0.0&amp;xxc=shop&amp;skuId=6133843852560</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=963160907330&amp;mi_id=0000texXRtofEsIzn9VdJIbr57lv5T0l3VRG4gfDk2BVmQc&amp;spm=a21xtw.29978516.0.0&amp;xxc=shop&amp;skuId=6069666995393</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=1080314843824&amp;mi_id=00006IJIU-IYDgQCHTmgH4dotuk_P6_dz4IpYEgD1dGJzXM&amp;spm=a21xtw.29978516.0.0&amp;xxc=shop&amp;skuId=6299301742939</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=982964565711&amp;mi_id=0000_kmn_oKVzMm048QP-6QoVRdcUFv8HXa-8SJ0qUFnkrc&amp;spm=a21xtw.29978516.0.0&amp;xxc=shop&amp;skuId=6108828551370</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=970351720471&amp;mi_id=00009XJxyR5eQnptp9oKHpwCdJk-1I-N0uR8ifLzjeAbxcs&amp;spm=a21xtw.29978516.0.0&amp;xxc=shop&amp;skuId=5918363197404</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=1078044637886&amp;mi_id=0000J87OeNLQxFOGILOF-Cmjr8xBRvuuQOhOTWvE4UBOEds&amp;spm=a21xtw.29978516.0.0&amp;xxc=shop&amp;skuId=6294096667192</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=1079411133222&amp;mi_id=0000w1OuQ1a-Nph0fojG5wOAAdYHmsfTexWgI4WspkWPjyY&amp;spm=a21xtw.29978516.0.0&amp;xxc=shop&amp;skuId=6295676018541</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=1080314063229&amp;mi_id=0000Zt3fqt7LEt7EReo8qhRbOjA5DBu7olECyjVOMPODw-8&amp;spm=a21xtw.29978516.0.0&amp;xxc=shop&amp;skuId=6299301358248</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=967752064868&amp;mi_id=0000CpL3azyK72rPccTNyTdhr7lqhwh2yfebBQiB9qIN-NE&amp;spm=a21xtw.29978516.0.0&amp;xxc=shop&amp;skuId=5913183157231</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=738083059484&amp;mi_id=0000ACRuZbzV72PT7o-iaU_Emu0wRmVKDC0FobF0rvobpJI&amp;spm=a21xtw.29978516.0.0&amp;xxc=shop&amp;skuId=5266998571770</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=1077843058059&amp;mi_id=0000rLkfn1yPoJSxZPfevD-wiotk4Fw7mp80gSWYvSGbTWo&amp;spm=a21xtw.29978516.0.0&amp;xxc=shop&amp;skuId=6294984198132</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=1081834756981&amp;mi_id=0000_w0jyA9LsQZQFeHPH58TnEFc0fblYp27HJZlamlATGM&amp;spm=a21xtw.29978516.0.0&amp;xxc=shop&amp;skuId=6297468266422</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=1076140587381&amp;mi_id=0000TMKrjFrxunsbgRkWBhL-0I3t-bzDMsCzF8FldykddzU&amp;spm=a21xtw.29978516.0.0&amp;xxc=shop&amp;skuId=6129113104002</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=1076689119808&amp;mi_id=00009sVKunp5SZGL0bD850jn8xXe-6gn2qiIEywMBBhWFdI&amp;spm=a21xtw.29978516.0.0&amp;xxc=shop&amp;skuId=6294863343539</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=1081837888025&amp;mi_id=00007eq3LGWe-K5mETtKlj5Bd8BVjolA8sYodLojNjh5Kec&amp;spm=a21xtw.29978516.0.0&amp;xxc=shop</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=1082130592462&amp;mi_id=0000rGXx964OHlJC0fnqKmsEoUTqDKxOmv1OtudhZxxOzO0&amp;spm=a21xtw.29978516.0.0&amp;xxc=shop</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=680877999136&amp;mi_id=0000gifhLscogikJRnwCdNqMCJyWBut4T0T250JOqtEJIlY&amp;spm=a21xtw.29978516.0.0&amp;xxc=shop</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=742216959144&amp;mi_id=0000lAhz9dQFEavS6N551DRgM6P8JDqLpEG50mePJfblTns&amp;spm=a21xtw.29978516.0.0&amp;xxc=shop</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=758951256874&amp;mi_id=0000GsPWnCUaPvmM_avKO8GIKX1mFfvbM5T7okfiG5w-XOY&amp;spm=a21xtw.29978516.0.0&amp;xxc=shop</t>
+  </si>
+  <si>
     <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_1077196468019</t>
   </si>
   <si>
@@ -248,6 +368,63 @@
   </si>
   <si>
     <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_1075294704720</t>
+  </si>
+  <si>
+    <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_1082717808296</t>
+  </si>
+  <si>
+    <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_963160907330</t>
+  </si>
+  <si>
+    <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_1080314843824</t>
+  </si>
+  <si>
+    <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_982964565711</t>
+  </si>
+  <si>
+    <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_970351720471</t>
+  </si>
+  <si>
+    <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_1078044637886</t>
+  </si>
+  <si>
+    <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_1079411133222</t>
+  </si>
+  <si>
+    <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_1080314063229</t>
+  </si>
+  <si>
+    <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_967752064868</t>
+  </si>
+  <si>
+    <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_738083059484</t>
+  </si>
+  <si>
+    <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_1077843058059</t>
+  </si>
+  <si>
+    <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_1081834756981</t>
+  </si>
+  <si>
+    <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_1076140587381</t>
+  </si>
+  <si>
+    <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_1076689119808</t>
+  </si>
+  <si>
+    <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_1081837888025</t>
+  </si>
+  <si>
+    <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_1082130592462</t>
+  </si>
+  <si>
+    <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_680877999136</t>
+  </si>
+  <si>
+    <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_742216959144</t>
+  </si>
+  <si>
+    <t>c:\Users\passp\Desktop\univercity\4-2\taobao_jackets\downloaded_jackets\item_758951256874</t>
   </si>
 </sst>
 </file>
@@ -618,7 +795,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -652,356 +829,736 @@
         <v>1077196468019</v>
       </c>
       <c r="C2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F2">
         <v>420</v>
       </c>
       <c r="G2" t="s">
-        <v>60</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
-        <v>7</v>
+      <c r="B3">
+        <v>811036195091</v>
       </c>
       <c r="C3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="F3">
         <v>150</v>
       </c>
       <c r="G3" t="s">
-        <v>61</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
-        <v>8</v>
+      <c r="B4">
+        <v>1080043211319</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="F4">
         <v>179</v>
       </c>
       <c r="G4" t="s">
-        <v>62</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5">
         <v>3</v>
       </c>
-      <c r="B5" t="s">
-        <v>9</v>
+      <c r="B5">
+        <v>1083932831050</v>
       </c>
       <c r="C5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>45</v>
+        <v>66</v>
       </c>
       <c r="F5">
         <v>164</v>
       </c>
       <c r="G5" t="s">
-        <v>63</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6">
         <v>4</v>
       </c>
-      <c r="B6" t="s">
-        <v>10</v>
+      <c r="B6">
+        <v>1071816497728</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="F6">
         <v>221</v>
       </c>
       <c r="G6" t="s">
-        <v>64</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7">
         <v>5</v>
       </c>
-      <c r="B7" t="s">
-        <v>11</v>
+      <c r="B7">
+        <v>1075139885104</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>47</v>
+        <v>68</v>
       </c>
       <c r="F7">
         <v>212</v>
       </c>
       <c r="G7" t="s">
-        <v>65</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8">
         <v>6</v>
       </c>
-      <c r="B8" t="s">
-        <v>12</v>
+      <c r="B8">
+        <v>1078567805117</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="F8">
         <v>213</v>
       </c>
       <c r="G8" t="s">
-        <v>66</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9">
         <v>7</v>
       </c>
-      <c r="B9" t="s">
-        <v>13</v>
+      <c r="B9">
+        <v>1061875162656</v>
       </c>
       <c r="C9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>49</v>
+        <v>70</v>
       </c>
       <c r="F9">
         <v>196</v>
       </c>
       <c r="G9" t="s">
-        <v>67</v>
+        <v>107</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10">
         <v>8</v>
       </c>
-      <c r="B10" t="s">
-        <v>14</v>
+      <c r="B10">
+        <v>1069955447343</v>
       </c>
       <c r="C10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>50</v>
+        <v>71</v>
       </c>
       <c r="F10">
         <v>203</v>
       </c>
       <c r="G10" t="s">
-        <v>68</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11">
         <v>9</v>
       </c>
-      <c r="B11" t="s">
-        <v>15</v>
+      <c r="B11">
+        <v>1075374113206</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>51</v>
+        <v>72</v>
       </c>
       <c r="F11">
         <v>177</v>
       </c>
       <c r="G11" t="s">
-        <v>69</v>
+        <v>109</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12">
         <v>10</v>
       </c>
-      <c r="B12" t="s">
-        <v>16</v>
+      <c r="B12">
+        <v>1081695145771</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="F12">
         <v>235</v>
       </c>
       <c r="G12" t="s">
-        <v>70</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13">
         <v>11</v>
       </c>
-      <c r="B13" t="s">
-        <v>17</v>
+      <c r="B13">
+        <v>1054456462690</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
       <c r="F13">
         <v>232</v>
       </c>
       <c r="G13" t="s">
-        <v>71</v>
+        <v>111</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14">
         <v>12</v>
       </c>
-      <c r="B14" t="s">
-        <v>18</v>
+      <c r="B14">
+        <v>1055642429134</v>
       </c>
       <c r="C14" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>54</v>
+        <v>75</v>
       </c>
       <c r="F14">
         <v>2</v>
       </c>
       <c r="G14" t="s">
-        <v>72</v>
+        <v>112</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15">
         <v>13</v>
       </c>
-      <c r="B15" t="s">
-        <v>19</v>
+      <c r="B15">
+        <v>1062441766322</v>
       </c>
       <c r="C15" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="F15">
         <v>2</v>
       </c>
       <c r="G15" t="s">
-        <v>73</v>
+        <v>113</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16">
         <v>14</v>
       </c>
-      <c r="B16" t="s">
-        <v>20</v>
+      <c r="B16">
+        <v>1071811849639</v>
       </c>
       <c r="C16" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>56</v>
+        <v>77</v>
       </c>
       <c r="F16">
         <v>2</v>
       </c>
       <c r="G16" t="s">
-        <v>74</v>
+        <v>114</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17">
         <v>15</v>
       </c>
-      <c r="B17" t="s">
-        <v>21</v>
+      <c r="B17">
+        <v>1073332440807</v>
       </c>
       <c r="C17" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="F17">
         <v>1</v>
       </c>
       <c r="G17" t="s">
-        <v>75</v>
+        <v>115</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18">
         <v>16</v>
       </c>
-      <c r="B18" t="s">
-        <v>22</v>
+      <c r="B18">
+        <v>1074826657600</v>
       </c>
       <c r="C18" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>58</v>
+        <v>79</v>
       </c>
       <c r="F18">
         <v>2</v>
       </c>
       <c r="G18" t="s">
-        <v>76</v>
+        <v>116</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19">
         <v>17</v>
       </c>
-      <c r="B19" t="s">
-        <v>23</v>
+      <c r="B19">
+        <v>1075294704720</v>
       </c>
       <c r="C19" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>59</v>
+        <v>80</v>
       </c>
       <c r="F19">
         <v>2</v>
       </c>
       <c r="G19" t="s">
-        <v>77</v>
+        <v>117</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20">
+        <v>1</v>
+      </c>
+      <c r="B20" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" t="s">
+        <v>44</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="F20">
+        <v>13</v>
+      </c>
+      <c r="G20" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21">
+        <v>2</v>
+      </c>
+      <c r="B21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" t="s">
+        <v>45</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="F21">
+        <v>15</v>
+      </c>
+      <c r="G21" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22">
+        <v>3</v>
+      </c>
+      <c r="B22" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" t="s">
+        <v>46</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F22">
+        <v>13</v>
+      </c>
+      <c r="G22" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23">
+        <v>4</v>
+      </c>
+      <c r="B23" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" t="s">
+        <v>47</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="F23">
+        <v>14</v>
+      </c>
+      <c r="G23" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24">
+        <v>5</v>
+      </c>
+      <c r="B24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C24" t="s">
+        <v>48</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F24">
+        <v>13</v>
+      </c>
+      <c r="G24" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25">
+        <v>6</v>
+      </c>
+      <c r="B25" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" t="s">
+        <v>49</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F25">
+        <v>14</v>
+      </c>
+      <c r="G25" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26">
+        <v>7</v>
+      </c>
+      <c r="B26" t="s">
+        <v>13</v>
+      </c>
+      <c r="C26" t="s">
+        <v>50</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="F26">
+        <v>13</v>
+      </c>
+      <c r="G26" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27">
+        <v>8</v>
+      </c>
+      <c r="B27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27" t="s">
+        <v>51</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F27">
+        <v>17</v>
+      </c>
+      <c r="G27" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28">
+        <v>9</v>
+      </c>
+      <c r="B28" t="s">
+        <v>15</v>
+      </c>
+      <c r="C28" t="s">
+        <v>52</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="F28">
+        <v>14</v>
+      </c>
+      <c r="G28" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29">
+        <v>10</v>
+      </c>
+      <c r="B29" t="s">
+        <v>16</v>
+      </c>
+      <c r="C29" t="s">
+        <v>53</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="F29">
+        <v>12</v>
+      </c>
+      <c r="G29" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30">
+        <v>11</v>
+      </c>
+      <c r="B30" t="s">
+        <v>17</v>
+      </c>
+      <c r="C30" t="s">
+        <v>54</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F30">
+        <v>17</v>
+      </c>
+      <c r="G30" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31">
+        <v>12</v>
+      </c>
+      <c r="B31" t="s">
+        <v>18</v>
+      </c>
+      <c r="C31" t="s">
+        <v>55</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="F31">
+        <v>13</v>
+      </c>
+      <c r="G31" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32">
+        <v>13</v>
+      </c>
+      <c r="B32" t="s">
+        <v>19</v>
+      </c>
+      <c r="C32" t="s">
+        <v>56</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="F32">
+        <v>14</v>
+      </c>
+      <c r="G32" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33">
+        <v>14</v>
+      </c>
+      <c r="B33" t="s">
+        <v>20</v>
+      </c>
+      <c r="C33" t="s">
+        <v>57</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F33">
+        <v>12</v>
+      </c>
+      <c r="G33" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34">
+        <v>15</v>
+      </c>
+      <c r="B34" t="s">
+        <v>21</v>
+      </c>
+      <c r="C34" t="s">
+        <v>58</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F34">
+        <v>2</v>
+      </c>
+      <c r="G34" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35">
+        <v>16</v>
+      </c>
+      <c r="B35" t="s">
+        <v>22</v>
+      </c>
+      <c r="C35" t="s">
+        <v>59</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="F35">
+        <v>2</v>
+      </c>
+      <c r="G35" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36">
+        <v>17</v>
+      </c>
+      <c r="B36" t="s">
+        <v>23</v>
+      </c>
+      <c r="C36" t="s">
+        <v>60</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="F36">
+        <v>2</v>
+      </c>
+      <c r="G36" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37">
+        <v>18</v>
+      </c>
+      <c r="B37" t="s">
+        <v>24</v>
+      </c>
+      <c r="C37" t="s">
+        <v>61</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="F37">
+        <v>2</v>
+      </c>
+      <c r="G37" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38">
+        <v>19</v>
+      </c>
+      <c r="B38" t="s">
+        <v>25</v>
+      </c>
+      <c r="C38" t="s">
+        <v>62</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="F38">
+        <v>2</v>
+      </c>
+      <c r="G38" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -1024,6 +1581,25 @@
     <hyperlink ref="E17" r:id="rId16"/>
     <hyperlink ref="E18" r:id="rId17"/>
     <hyperlink ref="E19" r:id="rId18"/>
+    <hyperlink ref="E20" r:id="rId19"/>
+    <hyperlink ref="E21" r:id="rId20"/>
+    <hyperlink ref="E22" r:id="rId21"/>
+    <hyperlink ref="E23" r:id="rId22"/>
+    <hyperlink ref="E24" r:id="rId23"/>
+    <hyperlink ref="E25" r:id="rId24"/>
+    <hyperlink ref="E26" r:id="rId25"/>
+    <hyperlink ref="E27" r:id="rId26"/>
+    <hyperlink ref="E28" r:id="rId27"/>
+    <hyperlink ref="E29" r:id="rId28"/>
+    <hyperlink ref="E30" r:id="rId29"/>
+    <hyperlink ref="E31" r:id="rId30"/>
+    <hyperlink ref="E32" r:id="rId31"/>
+    <hyperlink ref="E33" r:id="rId32"/>
+    <hyperlink ref="E34" r:id="rId33"/>
+    <hyperlink ref="E35" r:id="rId34"/>
+    <hyperlink ref="E36" r:id="rId35"/>
+    <hyperlink ref="E37" r:id="rId36"/>
+    <hyperlink ref="E38" r:id="rId37"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>